<commit_message>
Cleaned up public facing files
</commit_message>
<xml_diff>
--- a/Outputs/table_outputs.xlsx
+++ b/Outputs/table_outputs.xlsx
@@ -40,12 +40,24 @@
     <sheet name="Table S17a" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="Table S17b" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="Table S17c" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="Table S6 - city - USD" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="Table S6 - city - local" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="Table S6 - country - USD" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="Table S6 - country - local" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="Table S7 - city - USD" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="Table S7 - city - local" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="Table S8 - USD" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="Table S8 - local" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Table S7 - country - USD" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Table S7 - country - local" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="Table S7 - overall - USD" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="Table S7 - overall - local" sheetId="46" state="visible" r:id="rId46"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="1256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="1439">
   <si>
     <t xml:space="preserve">country</t>
   </si>
@@ -3813,6 +3825,555 @@
   </si>
   <si>
     <t xml:space="preserve">promo_theme_trad_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">median_org_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iqr_org_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min_org_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_org_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">median_conv_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iqr_conv_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min_conv_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_conv_rice_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.98 (1.76), 10.98-23.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.39 (1.66), 4.00-18.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.69 (0.00), 14.69-14.69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.90 (1.01), 1.90-8.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.25 (0.21), 4.99-5.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">83.50 (23.50), 60.00-107.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">107.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57.50 (10.00), 30.00-85.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.00 (10.00), 20.00-60.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.90 (25.00), 48.00-250.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">250.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.00 (13.50), 28.00-210.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">210.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.15 (0.55), 3.60-4.70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.40 (0.59), 0.55-4.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.55 (1.81), 3.06-10.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.87 (0.88), 0.45-6.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.99 (3.66), 4.05-10.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.36 (2.00), 1.40-7.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.98 (1.60), 10.98-23.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.90 (1.77), 1.90-18.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.77</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.90 (30.50), 48.00-250.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.00 (15.00), 20.00-210.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.80 (3.90), 3.06-10.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.42 (1.83), 0.45-7.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.83</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.98 (1.30), 10.98-23.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.75 (0.90), 4.58-7.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.89 (0.00), 5.89-5.89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">107.00 (0.00), 107.00-107.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68.00 (0.00), 68.00-68.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80.00 (35.00), 48.00-250.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64.00 (30.00), 38.00-102.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">102.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.45 (0.05), 2.40-2.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.50 (0.27), 3.06-3.60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.85 (0.10), 1.75-1.95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.49 (4.32), 4.19-10.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.35 (1.68), 1.52-6.85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">org_price_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conv_price_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.29 (5.46), 13.95-23.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.99 (3.18), 4.89-13.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.98 (0), 14.98-14.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.49 (1.5), 4-17.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.98 (0), 10.98-10.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 (3.19), 4.99-18.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.39 (1.66), 4-18.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.69 (0), 14.69-14.69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.89 (0), 5.89-5.89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.47 (0.95), 1.9-6.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.99 (1), 4.99-8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.9 (1.01), 1.9-8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.62 (0.28), 5.35-5.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.14 (0.13), 4.99-5.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.35 (0), 5.35-5.35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.25 (0.21), 4.99-5.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.98 (1.6), 10.98-23.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.9 (1.77), 1.9-18.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">83.5 (23.5), 60-107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57 (14.5), 40-85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57.5 (15), 30-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">55 (3), 50-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57.5 (10), 30-85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (8.75), 50-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45 (10), 35-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (0.75), 20-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (10), 20-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80 (85), 80-250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (15), 34-210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82.5 (30), 50-95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45.5 (10), 28-80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91.8 (49), 48-160</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (12.3), 36-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.9 (25), 48-250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (13.5), 28-210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.9 (30.5), 48-250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (15), 20-210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.15 (0.55), 3.6-4.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.45 (0.1), 1.7-4.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.22 (0.75), 1.4-3.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 (0.75), 0.55-4.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 (0.59), 0.55-4.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.8 (3.2), 3.6-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.38 (0.55), 1.35-3.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5 (0), 3.5-3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.68 (0.66), 0.45-3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.06 (0), 3.06-3.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8 (0.61), 0.45-6.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.55 (1.81), 3.06-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.87 (0.88), 0.45-6.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.98 (2.72), 4.05-9.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.17 (1.93), 1.4-7.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.49 (4.63), 4.38-10.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.79 (1.09), 2.15-5.69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.8 (1.9), 4.19-7.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.9 (2.21), 1.5-5.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.36 (2), 1.4-7.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.8 (3.9), 3.06-10.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.42 (1.83), 0.45-7.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.69 (63.02), 3.06-250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39 (45.01), 0.45-210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.84 (1.22), 10.98-23.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.75 (0.95), 4.58-7.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.90 (32.50), 48.00-250.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64.30 (27.00), 38.00-102.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.80 (4.08), 3.06-10.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.59 (1.69), 1.52-6.85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.99 (44.10), 3.06-250.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.69 (38.91), 1.52-102.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38.91</t>
   </si>
 </sst>
 </file>
@@ -21412,6 +21973,1429 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F1" t="s">
+        <v>415</v>
+      </c>
+      <c r="G1" t="s">
+        <v>416</v>
+      </c>
+      <c r="H1" t="s">
+        <v>417</v>
+      </c>
+      <c r="I1" t="s">
+        <v>418</v>
+      </c>
+      <c r="J1" t="s">
+        <v>419</v>
+      </c>
+      <c r="K1" t="s">
+        <v>420</v>
+      </c>
+      <c r="L1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D2" t="s">
+        <v>422</v>
+      </c>
+      <c r="E2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G2" t="s">
+        <v>425</v>
+      </c>
+      <c r="H2" t="s">
+        <v>426</v>
+      </c>
+      <c r="I2" t="s">
+        <v>427</v>
+      </c>
+      <c r="J2" t="s">
+        <v>428</v>
+      </c>
+      <c r="K2" t="s">
+        <v>429</v>
+      </c>
+      <c r="L2" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E3" t="s">
+        <v>431</v>
+      </c>
+      <c r="F3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G3" t="s">
+        <v>432</v>
+      </c>
+      <c r="H3" t="s">
+        <v>432</v>
+      </c>
+      <c r="I3" t="s">
+        <v>433</v>
+      </c>
+      <c r="J3" t="s">
+        <v>434</v>
+      </c>
+      <c r="K3" t="s">
+        <v>435</v>
+      </c>
+      <c r="L3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>271</v>
+      </c>
+      <c r="D4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E4" t="s">
+        <v>437</v>
+      </c>
+      <c r="F4" t="s">
+        <v>273</v>
+      </c>
+      <c r="G4" t="s">
+        <v>438</v>
+      </c>
+      <c r="H4" t="s">
+        <v>439</v>
+      </c>
+      <c r="I4" t="s">
+        <v>440</v>
+      </c>
+      <c r="J4" t="s">
+        <v>441</v>
+      </c>
+      <c r="K4" t="s">
+        <v>442</v>
+      </c>
+      <c r="L4" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D5" t="s">
+        <v>294</v>
+      </c>
+      <c r="E5" t="s">
+        <v>444</v>
+      </c>
+      <c r="F5" t="s">
+        <v>445</v>
+      </c>
+      <c r="G5" t="s">
+        <v>446</v>
+      </c>
+      <c r="H5" t="s">
+        <v>447</v>
+      </c>
+      <c r="I5" t="s">
+        <v>448</v>
+      </c>
+      <c r="J5" t="s">
+        <v>449</v>
+      </c>
+      <c r="K5" t="s">
+        <v>435</v>
+      </c>
+      <c r="L5" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>271</v>
+      </c>
+      <c r="D6" t="s">
+        <v>450</v>
+      </c>
+      <c r="E6" t="s">
+        <v>437</v>
+      </c>
+      <c r="F6" t="s">
+        <v>273</v>
+      </c>
+      <c r="G6" t="s">
+        <v>438</v>
+      </c>
+      <c r="H6" t="s">
+        <v>439</v>
+      </c>
+      <c r="I6" t="s">
+        <v>451</v>
+      </c>
+      <c r="J6" t="s">
+        <v>449</v>
+      </c>
+      <c r="K6" t="s">
+        <v>452</v>
+      </c>
+      <c r="L6" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" t="s">
+        <v>453</v>
+      </c>
+      <c r="D7" t="s">
+        <v>450</v>
+      </c>
+      <c r="E7" t="s">
+        <v>454</v>
+      </c>
+      <c r="F7" t="s">
+        <v>428</v>
+      </c>
+      <c r="G7" t="s">
+        <v>455</v>
+      </c>
+      <c r="H7" t="s">
+        <v>456</v>
+      </c>
+      <c r="I7" t="s">
+        <v>457</v>
+      </c>
+      <c r="J7" t="s">
+        <v>458</v>
+      </c>
+      <c r="K7" t="s">
+        <v>435</v>
+      </c>
+      <c r="L7" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>262</v>
+      </c>
+      <c r="D8" t="s">
+        <v>460</v>
+      </c>
+      <c r="E8" t="s">
+        <v>461</v>
+      </c>
+      <c r="F8" t="s">
+        <v>462</v>
+      </c>
+      <c r="G8" t="s">
+        <v>463</v>
+      </c>
+      <c r="H8" t="s">
+        <v>464</v>
+      </c>
+      <c r="I8" t="s">
+        <v>465</v>
+      </c>
+      <c r="J8" t="s">
+        <v>466</v>
+      </c>
+      <c r="K8" t="s">
+        <v>462</v>
+      </c>
+      <c r="L8" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
+        <v>254</v>
+      </c>
+      <c r="D9" t="s">
+        <v>468</v>
+      </c>
+      <c r="E9" t="s">
+        <v>469</v>
+      </c>
+      <c r="F9" t="s">
+        <v>470</v>
+      </c>
+      <c r="G9" t="s">
+        <v>471</v>
+      </c>
+      <c r="H9" t="s">
+        <v>472</v>
+      </c>
+      <c r="I9" t="s">
+        <v>473</v>
+      </c>
+      <c r="J9" t="s">
+        <v>301</v>
+      </c>
+      <c r="K9" t="s">
+        <v>474</v>
+      </c>
+      <c r="L9" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" t="s">
+        <v>289</v>
+      </c>
+      <c r="D10" t="s">
+        <v>476</v>
+      </c>
+      <c r="E10" t="s">
+        <v>477</v>
+      </c>
+      <c r="F10" t="s">
+        <v>478</v>
+      </c>
+      <c r="G10" t="s">
+        <v>479</v>
+      </c>
+      <c r="H10" t="s">
+        <v>480</v>
+      </c>
+      <c r="I10" t="s">
+        <v>481</v>
+      </c>
+      <c r="J10" t="s">
+        <v>482</v>
+      </c>
+      <c r="K10" t="s">
+        <v>436</v>
+      </c>
+      <c r="L10" t="s">
+        <v>483</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1257</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1260</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1261</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1262</v>
+      </c>
+      <c r="L1" t="s">
+        <v>1263</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D2" t="s">
+        <v>422</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1264</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1267</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1268</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1269</v>
+      </c>
+      <c r="K2" t="s">
+        <v>317</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="F3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1272</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1272</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1273</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1274</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1275</v>
+      </c>
+      <c r="L3" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>271</v>
+      </c>
+      <c r="D4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E4" t="s">
+        <v>437</v>
+      </c>
+      <c r="F4" t="s">
+        <v>273</v>
+      </c>
+      <c r="G4" t="s">
+        <v>438</v>
+      </c>
+      <c r="H4" t="s">
+        <v>439</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1277</v>
+      </c>
+      <c r="J4" t="s">
+        <v>434</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1278</v>
+      </c>
+      <c r="L4" t="s">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D5" t="s">
+        <v>294</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1280</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1281</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1282</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1283</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J5" t="s">
+        <v>1285</v>
+      </c>
+      <c r="K5" t="s">
+        <v>1286</v>
+      </c>
+      <c r="L5" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>271</v>
+      </c>
+      <c r="D6" t="s">
+        <v>450</v>
+      </c>
+      <c r="E6" t="s">
+        <v>437</v>
+      </c>
+      <c r="F6" t="s">
+        <v>273</v>
+      </c>
+      <c r="G6" t="s">
+        <v>438</v>
+      </c>
+      <c r="H6" t="s">
+        <v>439</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1288</v>
+      </c>
+      <c r="J6" t="s">
+        <v>1285</v>
+      </c>
+      <c r="K6" t="s">
+        <v>1289</v>
+      </c>
+      <c r="L6" t="s">
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" t="s">
+        <v>453</v>
+      </c>
+      <c r="D7" t="s">
+        <v>450</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1290</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1291</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1292</v>
+      </c>
+      <c r="H7" t="s">
+        <v>1293</v>
+      </c>
+      <c r="I7" t="s">
+        <v>1294</v>
+      </c>
+      <c r="J7" t="s">
+        <v>1295</v>
+      </c>
+      <c r="K7" t="s">
+        <v>1296</v>
+      </c>
+      <c r="L7" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>262</v>
+      </c>
+      <c r="D8" t="s">
+        <v>460</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1299</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1300</v>
+      </c>
+      <c r="H8" t="s">
+        <v>1301</v>
+      </c>
+      <c r="I8" t="s">
+        <v>1302</v>
+      </c>
+      <c r="J8" t="s">
+        <v>1303</v>
+      </c>
+      <c r="K8" t="s">
+        <v>1299</v>
+      </c>
+      <c r="L8" t="s">
+        <v>1304</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
+        <v>254</v>
+      </c>
+      <c r="D9" t="s">
+        <v>468</v>
+      </c>
+      <c r="E9" t="s">
+        <v>1305</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1306</v>
+      </c>
+      <c r="G9" t="s">
+        <v>1307</v>
+      </c>
+      <c r="H9" t="s">
+        <v>1285</v>
+      </c>
+      <c r="I9" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J9" t="s">
+        <v>509</v>
+      </c>
+      <c r="K9" t="s">
+        <v>517</v>
+      </c>
+      <c r="L9" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" t="s">
+        <v>289</v>
+      </c>
+      <c r="D10" t="s">
+        <v>476</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1310</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1311</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1312</v>
+      </c>
+      <c r="H10" t="s">
+        <v>1313</v>
+      </c>
+      <c r="I10" t="s">
+        <v>1314</v>
+      </c>
+      <c r="J10" t="s">
+        <v>270</v>
+      </c>
+      <c r="K10" t="s">
+        <v>1315</v>
+      </c>
+      <c r="L10" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D1" t="s">
+        <v>414</v>
+      </c>
+      <c r="E1" t="s">
+        <v>415</v>
+      </c>
+      <c r="F1" t="s">
+        <v>416</v>
+      </c>
+      <c r="G1" t="s">
+        <v>417</v>
+      </c>
+      <c r="H1" t="s">
+        <v>418</v>
+      </c>
+      <c r="I1" t="s">
+        <v>419</v>
+      </c>
+      <c r="J1" t="s">
+        <v>420</v>
+      </c>
+      <c r="K1" t="s">
+        <v>421</v>
+      </c>
+      <c r="L1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C2" t="s">
+        <v>485</v>
+      </c>
+      <c r="D2" t="s">
+        <v>486</v>
+      </c>
+      <c r="E2" t="s">
+        <v>487</v>
+      </c>
+      <c r="F2" t="s">
+        <v>425</v>
+      </c>
+      <c r="G2" t="s">
+        <v>426</v>
+      </c>
+      <c r="H2" t="s">
+        <v>488</v>
+      </c>
+      <c r="I2" t="s">
+        <v>489</v>
+      </c>
+      <c r="J2" t="s">
+        <v>435</v>
+      </c>
+      <c r="K2" t="s">
+        <v>430</v>
+      </c>
+      <c r="L2" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>491</v>
+      </c>
+      <c r="C3" t="s">
+        <v>492</v>
+      </c>
+      <c r="D3" t="s">
+        <v>493</v>
+      </c>
+      <c r="E3" t="s">
+        <v>494</v>
+      </c>
+      <c r="F3" t="s">
+        <v>455</v>
+      </c>
+      <c r="G3" t="s">
+        <v>456</v>
+      </c>
+      <c r="H3" t="s">
+        <v>495</v>
+      </c>
+      <c r="I3" t="s">
+        <v>496</v>
+      </c>
+      <c r="J3" t="s">
+        <v>452</v>
+      </c>
+      <c r="K3" t="s">
+        <v>459</v>
+      </c>
+      <c r="L3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C4" t="s">
+        <v>497</v>
+      </c>
+      <c r="D4" t="s">
+        <v>498</v>
+      </c>
+      <c r="E4" t="s">
+        <v>499</v>
+      </c>
+      <c r="F4" t="s">
+        <v>471</v>
+      </c>
+      <c r="G4" t="s">
+        <v>480</v>
+      </c>
+      <c r="H4" t="s">
+        <v>500</v>
+      </c>
+      <c r="I4" t="s">
+        <v>501</v>
+      </c>
+      <c r="J4" t="s">
+        <v>474</v>
+      </c>
+      <c r="K4" t="s">
+        <v>483</v>
+      </c>
+      <c r="L4" t="s">
+        <v>490</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1256</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1257</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1260</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1261</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1262</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1263</v>
+      </c>
+      <c r="L1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C2" t="s">
+        <v>485</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1317</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1267</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1319</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1320</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1275</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1270</v>
+      </c>
+      <c r="L2" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>491</v>
+      </c>
+      <c r="C3" t="s">
+        <v>492</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1321</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1322</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1292</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1323</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1324</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1289</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1297</v>
+      </c>
+      <c r="L3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C4" t="s">
+        <v>497</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1326</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1307</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1327</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1328</v>
+      </c>
+      <c r="J4" t="s">
+        <v>517</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1316</v>
+      </c>
+      <c r="L4" t="s">
+        <v>490</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F1" t="s">
+        <v>415</v>
+      </c>
+      <c r="G1" t="s">
+        <v>416</v>
+      </c>
+      <c r="H1" t="s">
+        <v>417</v>
+      </c>
+      <c r="I1" t="s">
+        <v>418</v>
+      </c>
+      <c r="J1" t="s">
+        <v>419</v>
+      </c>
+      <c r="K1" t="s">
+        <v>420</v>
+      </c>
+      <c r="L1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E2" t="s">
+        <v>507</v>
+      </c>
+      <c r="F2" t="s">
+        <v>327</v>
+      </c>
+      <c r="G2" t="s">
+        <v>425</v>
+      </c>
+      <c r="H2" t="s">
+        <v>426</v>
+      </c>
+      <c r="I2" t="s">
+        <v>508</v>
+      </c>
+      <c r="J2" t="s">
+        <v>458</v>
+      </c>
+      <c r="K2" t="s">
+        <v>509</v>
+      </c>
+      <c r="L2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D3" t="s">
+        <v>267</v>
+      </c>
+      <c r="E3" t="s">
+        <v>431</v>
+      </c>
+      <c r="F3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G3" t="s">
+        <v>432</v>
+      </c>
+      <c r="H3" t="s">
+        <v>432</v>
+      </c>
+      <c r="I3" t="s">
+        <v>511</v>
+      </c>
+      <c r="J3" t="s">
+        <v>258</v>
+      </c>
+      <c r="K3" t="s">
+        <v>512</v>
+      </c>
+      <c r="L3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>267</v>
+      </c>
+      <c r="D4" t="s">
+        <v>267</v>
+      </c>
+      <c r="E4" t="s">
+        <v>513</v>
+      </c>
+      <c r="F4" t="s">
+        <v>258</v>
+      </c>
+      <c r="G4" t="s">
+        <v>447</v>
+      </c>
+      <c r="H4" t="s">
+        <v>447</v>
+      </c>
+      <c r="I4" t="s">
+        <v>514</v>
+      </c>
+      <c r="J4" t="s">
+        <v>258</v>
+      </c>
+      <c r="K4" t="s">
+        <v>515</v>
+      </c>
+      <c r="L4" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E5" t="s">
+        <v>516</v>
+      </c>
+      <c r="F5" t="s">
+        <v>517</v>
+      </c>
+      <c r="G5" t="s">
+        <v>455</v>
+      </c>
+      <c r="H5" t="s">
+        <v>456</v>
+      </c>
+      <c r="I5" t="s">
+        <v>518</v>
+      </c>
+      <c r="J5" t="s">
+        <v>519</v>
+      </c>
+      <c r="K5" t="s">
+        <v>520</v>
+      </c>
+      <c r="L5" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>262</v>
+      </c>
+      <c r="D6" t="s">
+        <v>262</v>
+      </c>
+      <c r="E6" t="s">
+        <v>461</v>
+      </c>
+      <c r="F6" t="s">
+        <v>462</v>
+      </c>
+      <c r="G6" t="s">
+        <v>463</v>
+      </c>
+      <c r="H6" t="s">
+        <v>464</v>
+      </c>
+      <c r="I6" t="s">
+        <v>522</v>
+      </c>
+      <c r="J6" t="s">
+        <v>523</v>
+      </c>
+      <c r="K6" t="s">
+        <v>524</v>
+      </c>
+      <c r="L6" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
+        <v>526</v>
+      </c>
+      <c r="D7" t="s">
+        <v>526</v>
+      </c>
+      <c r="E7" t="s">
+        <v>527</v>
+      </c>
+      <c r="F7" t="s">
+        <v>487</v>
+      </c>
+      <c r="G7" t="s">
+        <v>471</v>
+      </c>
+      <c r="H7" t="s">
+        <v>528</v>
+      </c>
+      <c r="I7" t="s">
+        <v>529</v>
+      </c>
+      <c r="J7" t="s">
+        <v>530</v>
+      </c>
+      <c r="K7" t="s">
+        <v>531</v>
+      </c>
+      <c r="L7" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>285</v>
+      </c>
+      <c r="D8" t="s">
+        <v>285</v>
+      </c>
+      <c r="E8" t="s">
+        <v>533</v>
+      </c>
+      <c r="F8" t="s">
+        <v>534</v>
+      </c>
+      <c r="G8" t="s">
+        <v>535</v>
+      </c>
+      <c r="H8" t="s">
+        <v>480</v>
+      </c>
+      <c r="I8" t="s">
+        <v>536</v>
+      </c>
+      <c r="J8" t="s">
+        <v>537</v>
+      </c>
+      <c r="K8" t="s">
+        <v>538</v>
+      </c>
+      <c r="L8" t="s">
+        <v>539</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -21615,6 +23599,2879 @@
       </c>
       <c r="F10" t="n">
         <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1257</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1260</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1261</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1262</v>
+      </c>
+      <c r="L1" t="s">
+        <v>1263</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1329</v>
+      </c>
+      <c r="F2" t="s">
+        <v>447</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1267</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1330</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1331</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1332</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D3" t="s">
+        <v>267</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="F3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1272</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1272</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1334</v>
+      </c>
+      <c r="J3" t="s">
+        <v>258</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1335</v>
+      </c>
+      <c r="L3" t="s">
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>267</v>
+      </c>
+      <c r="D4" t="s">
+        <v>267</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1336</v>
+      </c>
+      <c r="F4" t="s">
+        <v>258</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="J4" t="s">
+        <v>258</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="L4" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1339</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1340</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1292</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1293</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1341</v>
+      </c>
+      <c r="J5" t="s">
+        <v>1286</v>
+      </c>
+      <c r="K5" t="s">
+        <v>1342</v>
+      </c>
+      <c r="L5" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>262</v>
+      </c>
+      <c r="D6" t="s">
+        <v>262</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1299</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1300</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1301</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1344</v>
+      </c>
+      <c r="J6" t="s">
+        <v>1345</v>
+      </c>
+      <c r="K6" t="s">
+        <v>1346</v>
+      </c>
+      <c r="L6" t="s">
+        <v>1347</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
+        <v>526</v>
+      </c>
+      <c r="D7" t="s">
+        <v>526</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1348</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1349</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1307</v>
+      </c>
+      <c r="H7" t="s">
+        <v>1300</v>
+      </c>
+      <c r="I7" t="s">
+        <v>1350</v>
+      </c>
+      <c r="J7" t="s">
+        <v>1351</v>
+      </c>
+      <c r="K7" t="s">
+        <v>1352</v>
+      </c>
+      <c r="L7" t="s">
+        <v>1353</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>285</v>
+      </c>
+      <c r="D8" t="s">
+        <v>285</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1354</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1355</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1356</v>
+      </c>
+      <c r="H8" t="s">
+        <v>1313</v>
+      </c>
+      <c r="I8" t="s">
+        <v>1357</v>
+      </c>
+      <c r="J8" t="s">
+        <v>1358</v>
+      </c>
+      <c r="K8" t="s">
+        <v>1359</v>
+      </c>
+      <c r="L8" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" t="s">
+        <v>412</v>
+      </c>
+      <c r="E1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F1" t="s">
+        <v>557</v>
+      </c>
+      <c r="G1" t="s">
+        <v>558</v>
+      </c>
+      <c r="H1" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>560</v>
+      </c>
+      <c r="G2" t="s">
+        <v>561</v>
+      </c>
+      <c r="H2" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>563</v>
+      </c>
+      <c r="G3" t="s">
+        <v>564</v>
+      </c>
+      <c r="H3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>565</v>
+      </c>
+      <c r="G4" t="s">
+        <v>566</v>
+      </c>
+      <c r="H4" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F5" t="s">
+        <v>423</v>
+      </c>
+      <c r="G5" t="s">
+        <v>427</v>
+      </c>
+      <c r="H5" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>568</v>
+      </c>
+      <c r="G6" t="s">
+        <v>569</v>
+      </c>
+      <c r="H6" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>570</v>
+      </c>
+      <c r="G7" t="s">
+        <v>571</v>
+      </c>
+      <c r="H7" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>570</v>
+      </c>
+      <c r="G8" t="s">
+        <v>572</v>
+      </c>
+      <c r="H8" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9"/>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>568</v>
+      </c>
+      <c r="G9" t="s">
+        <v>433</v>
+      </c>
+      <c r="H9" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="s">
+        <v>570</v>
+      </c>
+      <c r="G10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H10" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>570</v>
+      </c>
+      <c r="G11" t="s">
+        <v>574</v>
+      </c>
+      <c r="H11" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>570</v>
+      </c>
+      <c r="G12" t="s">
+        <v>575</v>
+      </c>
+      <c r="H12" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>7</v>
+      </c>
+      <c r="F13" t="s">
+        <v>570</v>
+      </c>
+      <c r="G13" t="s">
+        <v>440</v>
+      </c>
+      <c r="H13" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14" t="n">
+        <v>11</v>
+      </c>
+      <c r="E14" t="n">
+        <v>79</v>
+      </c>
+      <c r="F14" t="s">
+        <v>486</v>
+      </c>
+      <c r="G14" t="s">
+        <v>576</v>
+      </c>
+      <c r="H14" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" t="s">
+        <v>578</v>
+      </c>
+      <c r="G15" t="s">
+        <v>579</v>
+      </c>
+      <c r="H15" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s">
+        <v>570</v>
+      </c>
+      <c r="G16" t="s">
+        <v>580</v>
+      </c>
+      <c r="H16" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F17" t="s">
+        <v>570</v>
+      </c>
+      <c r="G17" t="s">
+        <v>581</v>
+      </c>
+      <c r="H17" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18"/>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>59</v>
+      </c>
+      <c r="F18" t="s">
+        <v>578</v>
+      </c>
+      <c r="G18" t="s">
+        <v>448</v>
+      </c>
+      <c r="H18" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" t="s">
+        <v>570</v>
+      </c>
+      <c r="G19" t="s">
+        <v>582</v>
+      </c>
+      <c r="H19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>44</v>
+      </c>
+      <c r="F20" t="s">
+        <v>570</v>
+      </c>
+      <c r="G20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H20" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>20</v>
+      </c>
+      <c r="F21" t="s">
+        <v>570</v>
+      </c>
+      <c r="G21" t="s">
+        <v>584</v>
+      </c>
+      <c r="H21" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22"/>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>74</v>
+      </c>
+      <c r="F22" t="s">
+        <v>570</v>
+      </c>
+      <c r="G22" t="s">
+        <v>451</v>
+      </c>
+      <c r="H22" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="s">
+        <v>99</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>31</v>
+      </c>
+      <c r="F23" t="s">
+        <v>585</v>
+      </c>
+      <c r="G23" t="s">
+        <v>586</v>
+      </c>
+      <c r="H23" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28</v>
+      </c>
+      <c r="F24" t="s">
+        <v>587</v>
+      </c>
+      <c r="G24" t="s">
+        <v>588</v>
+      </c>
+      <c r="H24" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D25" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" t="s">
+        <v>589</v>
+      </c>
+      <c r="G25" t="s">
+        <v>590</v>
+      </c>
+      <c r="H25" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26"/>
+      <c r="D26" t="n">
+        <v>14</v>
+      </c>
+      <c r="E26" t="n">
+        <v>74</v>
+      </c>
+      <c r="F26" t="s">
+        <v>591</v>
+      </c>
+      <c r="G26" t="s">
+        <v>457</v>
+      </c>
+      <c r="H26" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27"/>
+      <c r="C27"/>
+      <c r="D27" t="n">
+        <v>16</v>
+      </c>
+      <c r="E27" t="n">
+        <v>207</v>
+      </c>
+      <c r="F27" t="s">
+        <v>592</v>
+      </c>
+      <c r="G27" t="s">
+        <v>495</v>
+      </c>
+      <c r="H27" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="s">
+        <v>461</v>
+      </c>
+      <c r="G28" t="s">
+        <v>593</v>
+      </c>
+      <c r="H28" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" t="s">
+        <v>105</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>570</v>
+      </c>
+      <c r="G29" t="s">
+        <v>594</v>
+      </c>
+      <c r="H29" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" t="s">
+        <v>102</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>570</v>
+      </c>
+      <c r="G30" t="s">
+        <v>595</v>
+      </c>
+      <c r="H30" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31"/>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>25</v>
+      </c>
+      <c r="F31" t="s">
+        <v>461</v>
+      </c>
+      <c r="G31" t="s">
+        <v>465</v>
+      </c>
+      <c r="H31" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" t="s">
+        <v>99</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="s">
+        <v>596</v>
+      </c>
+      <c r="G32" t="s">
+        <v>597</v>
+      </c>
+      <c r="H32" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>598</v>
+      </c>
+      <c r="G33" t="s">
+        <v>599</v>
+      </c>
+      <c r="H33" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" t="s">
+        <v>102</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" t="s">
+        <v>600</v>
+      </c>
+      <c r="G34" t="s">
+        <v>601</v>
+      </c>
+      <c r="H34" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35"/>
+      <c r="D35" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" t="n">
+        <v>28</v>
+      </c>
+      <c r="F35" t="s">
+        <v>469</v>
+      </c>
+      <c r="G35" t="s">
+        <v>602</v>
+      </c>
+      <c r="H35" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>99</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>603</v>
+      </c>
+      <c r="G36" t="s">
+        <v>604</v>
+      </c>
+      <c r="H36" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" t="n">
+        <v>6</v>
+      </c>
+      <c r="E37" t="n">
+        <v>10</v>
+      </c>
+      <c r="F37" t="s">
+        <v>605</v>
+      </c>
+      <c r="G37" t="s">
+        <v>606</v>
+      </c>
+      <c r="H37" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" t="s">
+        <v>102</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" t="n">
+        <v>15</v>
+      </c>
+      <c r="F38" t="s">
+        <v>607</v>
+      </c>
+      <c r="G38" t="s">
+        <v>608</v>
+      </c>
+      <c r="H38" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39"/>
+      <c r="D39" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" t="n">
+        <v>39</v>
+      </c>
+      <c r="F39" t="s">
+        <v>609</v>
+      </c>
+      <c r="G39" t="s">
+        <v>610</v>
+      </c>
+      <c r="H39" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E40" t="n">
+        <v>92</v>
+      </c>
+      <c r="F40" t="s">
+        <v>498</v>
+      </c>
+      <c r="G40" t="s">
+        <v>611</v>
+      </c>
+      <c r="H40" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41"/>
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41" t="n">
+        <v>45</v>
+      </c>
+      <c r="E41" t="n">
+        <v>378</v>
+      </c>
+      <c r="F41" t="s">
+        <v>504</v>
+      </c>
+      <c r="G41" t="s">
+        <v>612</v>
+      </c>
+      <c r="H41" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" t="s">
+        <v>412</v>
+      </c>
+      <c r="E1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1361</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1362</v>
+      </c>
+      <c r="H1" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1363</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1364</v>
+      </c>
+      <c r="H2" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1365</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1366</v>
+      </c>
+      <c r="H3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1367</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1368</v>
+      </c>
+      <c r="H4" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1264</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1369</v>
+      </c>
+      <c r="H5" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1370</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1371</v>
+      </c>
+      <c r="H6" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>570</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1372</v>
+      </c>
+      <c r="H7" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>570</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1373</v>
+      </c>
+      <c r="H8" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9"/>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1370</v>
+      </c>
+      <c r="G9" t="s">
+        <v>1374</v>
+      </c>
+      <c r="H9" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="s">
+        <v>570</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1375</v>
+      </c>
+      <c r="H10" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>570</v>
+      </c>
+      <c r="G11" t="s">
+        <v>1376</v>
+      </c>
+      <c r="H11" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>570</v>
+      </c>
+      <c r="G12" t="s">
+        <v>1377</v>
+      </c>
+      <c r="H12" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>7</v>
+      </c>
+      <c r="F13" t="s">
+        <v>570</v>
+      </c>
+      <c r="G13" t="s">
+        <v>1378</v>
+      </c>
+      <c r="H13" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14" t="n">
+        <v>11</v>
+      </c>
+      <c r="E14" t="n">
+        <v>79</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1379</v>
+      </c>
+      <c r="G14" t="s">
+        <v>1380</v>
+      </c>
+      <c r="H14" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1381</v>
+      </c>
+      <c r="G15" t="s">
+        <v>1382</v>
+      </c>
+      <c r="H15" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s">
+        <v>570</v>
+      </c>
+      <c r="G16" t="s">
+        <v>1383</v>
+      </c>
+      <c r="H16" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F17" t="s">
+        <v>570</v>
+      </c>
+      <c r="G17" t="s">
+        <v>1384</v>
+      </c>
+      <c r="H17" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18"/>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>59</v>
+      </c>
+      <c r="F18" t="s">
+        <v>1381</v>
+      </c>
+      <c r="G18" t="s">
+        <v>1385</v>
+      </c>
+      <c r="H18" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" t="s">
+        <v>570</v>
+      </c>
+      <c r="G19" t="s">
+        <v>1386</v>
+      </c>
+      <c r="H19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>44</v>
+      </c>
+      <c r="F20" t="s">
+        <v>570</v>
+      </c>
+      <c r="G20" t="s">
+        <v>1387</v>
+      </c>
+      <c r="H20" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>20</v>
+      </c>
+      <c r="F21" t="s">
+        <v>570</v>
+      </c>
+      <c r="G21" t="s">
+        <v>1388</v>
+      </c>
+      <c r="H21" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22"/>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>74</v>
+      </c>
+      <c r="F22" t="s">
+        <v>570</v>
+      </c>
+      <c r="G22" t="s">
+        <v>1389</v>
+      </c>
+      <c r="H22" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="s">
+        <v>99</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>31</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1390</v>
+      </c>
+      <c r="G23" t="s">
+        <v>1391</v>
+      </c>
+      <c r="H23" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28</v>
+      </c>
+      <c r="F24" t="s">
+        <v>1392</v>
+      </c>
+      <c r="G24" t="s">
+        <v>1393</v>
+      </c>
+      <c r="H24" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D25" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1394</v>
+      </c>
+      <c r="G25" t="s">
+        <v>1395</v>
+      </c>
+      <c r="H25" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26"/>
+      <c r="D26" t="n">
+        <v>14</v>
+      </c>
+      <c r="E26" t="n">
+        <v>74</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1396</v>
+      </c>
+      <c r="G26" t="s">
+        <v>1397</v>
+      </c>
+      <c r="H26" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27"/>
+      <c r="C27"/>
+      <c r="D27" t="n">
+        <v>16</v>
+      </c>
+      <c r="E27" t="n">
+        <v>207</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1398</v>
+      </c>
+      <c r="G27" t="s">
+        <v>1399</v>
+      </c>
+      <c r="H27" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="s">
+        <v>1400</v>
+      </c>
+      <c r="G28" t="s">
+        <v>1401</v>
+      </c>
+      <c r="H28" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" t="s">
+        <v>105</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>570</v>
+      </c>
+      <c r="G29" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H29" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" t="s">
+        <v>102</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>570</v>
+      </c>
+      <c r="G30" t="s">
+        <v>1403</v>
+      </c>
+      <c r="H30" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31"/>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>25</v>
+      </c>
+      <c r="F31" t="s">
+        <v>1400</v>
+      </c>
+      <c r="G31" t="s">
+        <v>1404</v>
+      </c>
+      <c r="H31" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" t="s">
+        <v>99</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1405</v>
+      </c>
+      <c r="G32" t="s">
+        <v>1406</v>
+      </c>
+      <c r="H32" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1407</v>
+      </c>
+      <c r="G33" t="s">
+        <v>1408</v>
+      </c>
+      <c r="H33" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" t="s">
+        <v>102</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" t="s">
+        <v>1409</v>
+      </c>
+      <c r="G34" t="s">
+        <v>1410</v>
+      </c>
+      <c r="H34" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35"/>
+      <c r="D35" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" t="n">
+        <v>28</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1411</v>
+      </c>
+      <c r="G35" t="s">
+        <v>1412</v>
+      </c>
+      <c r="H35" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>99</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1413</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1414</v>
+      </c>
+      <c r="H36" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" t="n">
+        <v>6</v>
+      </c>
+      <c r="E37" t="n">
+        <v>10</v>
+      </c>
+      <c r="F37" t="s">
+        <v>1415</v>
+      </c>
+      <c r="G37" t="s">
+        <v>1416</v>
+      </c>
+      <c r="H37" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" t="s">
+        <v>102</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" t="n">
+        <v>15</v>
+      </c>
+      <c r="F38" t="s">
+        <v>1417</v>
+      </c>
+      <c r="G38" t="s">
+        <v>1418</v>
+      </c>
+      <c r="H38" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39"/>
+      <c r="D39" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" t="n">
+        <v>39</v>
+      </c>
+      <c r="F39" t="s">
+        <v>1310</v>
+      </c>
+      <c r="G39" t="s">
+        <v>1419</v>
+      </c>
+      <c r="H39" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E40" t="n">
+        <v>92</v>
+      </c>
+      <c r="F40" t="s">
+        <v>1420</v>
+      </c>
+      <c r="G40" t="s">
+        <v>1421</v>
+      </c>
+      <c r="H40" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41"/>
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41" t="n">
+        <v>45</v>
+      </c>
+      <c r="E41" t="n">
+        <v>378</v>
+      </c>
+      <c r="F41" t="s">
+        <v>1422</v>
+      </c>
+      <c r="G41" t="s">
+        <v>1423</v>
+      </c>
+      <c r="H41" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D1" t="s">
+        <v>414</v>
+      </c>
+      <c r="E1" t="s">
+        <v>415</v>
+      </c>
+      <c r="F1" t="s">
+        <v>416</v>
+      </c>
+      <c r="G1" t="s">
+        <v>417</v>
+      </c>
+      <c r="H1" t="s">
+        <v>418</v>
+      </c>
+      <c r="I1" t="s">
+        <v>419</v>
+      </c>
+      <c r="J1" t="s">
+        <v>420</v>
+      </c>
+      <c r="K1" t="s">
+        <v>421</v>
+      </c>
+      <c r="L1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D2" t="s">
+        <v>540</v>
+      </c>
+      <c r="E2" t="s">
+        <v>541</v>
+      </c>
+      <c r="F2" t="s">
+        <v>425</v>
+      </c>
+      <c r="G2" t="s">
+        <v>426</v>
+      </c>
+      <c r="H2" t="s">
+        <v>542</v>
+      </c>
+      <c r="I2" t="s">
+        <v>496</v>
+      </c>
+      <c r="J2" t="s">
+        <v>509</v>
+      </c>
+      <c r="K2" t="s">
+        <v>510</v>
+      </c>
+      <c r="L2" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>285</v>
+      </c>
+      <c r="C3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D3" t="s">
+        <v>543</v>
+      </c>
+      <c r="E3" t="s">
+        <v>544</v>
+      </c>
+      <c r="F3" t="s">
+        <v>455</v>
+      </c>
+      <c r="G3" t="s">
+        <v>456</v>
+      </c>
+      <c r="H3" t="s">
+        <v>545</v>
+      </c>
+      <c r="I3" t="s">
+        <v>546</v>
+      </c>
+      <c r="J3" t="s">
+        <v>520</v>
+      </c>
+      <c r="K3" t="s">
+        <v>521</v>
+      </c>
+      <c r="L3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>547</v>
+      </c>
+      <c r="C4" t="s">
+        <v>547</v>
+      </c>
+      <c r="D4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E4" t="s">
+        <v>549</v>
+      </c>
+      <c r="F4" t="s">
+        <v>471</v>
+      </c>
+      <c r="G4" t="s">
+        <v>480</v>
+      </c>
+      <c r="H4" t="s">
+        <v>550</v>
+      </c>
+      <c r="I4" t="s">
+        <v>551</v>
+      </c>
+      <c r="J4" t="s">
+        <v>538</v>
+      </c>
+      <c r="K4" t="s">
+        <v>539</v>
+      </c>
+      <c r="L4" t="s">
+        <v>490</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1256</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1257</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1260</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1261</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1262</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1263</v>
+      </c>
+      <c r="L1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1424</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1425</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1267</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1426</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1427</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1332</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1333</v>
+      </c>
+      <c r="L2" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>285</v>
+      </c>
+      <c r="C3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1428</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1429</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1292</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1430</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1431</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1342</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1343</v>
+      </c>
+      <c r="L3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>547</v>
+      </c>
+      <c r="C4" t="s">
+        <v>547</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1432</v>
+      </c>
+      <c r="E4" t="s">
+        <v>528</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1307</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1433</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1434</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1360</v>
+      </c>
+      <c r="L4" t="s">
+        <v>490</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" t="s">
+        <v>414</v>
+      </c>
+      <c r="D1" t="s">
+        <v>415</v>
+      </c>
+      <c r="E1" t="s">
+        <v>416</v>
+      </c>
+      <c r="F1" t="s">
+        <v>417</v>
+      </c>
+      <c r="G1" t="s">
+        <v>418</v>
+      </c>
+      <c r="H1" t="s">
+        <v>419</v>
+      </c>
+      <c r="I1" t="s">
+        <v>420</v>
+      </c>
+      <c r="J1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>552</v>
+      </c>
+      <c r="B2" t="s">
+        <v>552</v>
+      </c>
+      <c r="C2" t="s">
+        <v>553</v>
+      </c>
+      <c r="D2" t="s">
+        <v>554</v>
+      </c>
+      <c r="E2" t="s">
+        <v>455</v>
+      </c>
+      <c r="F2" t="s">
+        <v>480</v>
+      </c>
+      <c r="G2" t="s">
+        <v>555</v>
+      </c>
+      <c r="H2" t="s">
+        <v>556</v>
+      </c>
+      <c r="I2" t="s">
+        <v>520</v>
+      </c>
+      <c r="J2" t="s">
+        <v>539</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1256</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1257</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1260</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1261</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1262</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1263</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>552</v>
+      </c>
+      <c r="B2" t="s">
+        <v>552</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1435</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1436</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1307</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1293</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1437</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1438</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1359</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>